<commit_message>
Apply AlphaForge patch: alpha_forge_v4_premium_ui_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Insights.xlsx
+++ b/AlphaForge_Insights.xlsx
@@ -755,7 +755,7 @@
         <v>79.3</v>
       </c>
       <c r="G2" t="n">
-        <v>79.59999999999999</v>
+        <v>79.7</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -788,10 +788,10 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>16.3</v>
+        <v>16.09</v>
       </c>
       <c r="O2" t="n">
-        <v>43.12</v>
+        <v>42.87</v>
       </c>
       <c r="P2" t="n">
         <v>16.01</v>
@@ -803,7 +803,7 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Buy Watchlist, score 79.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 5.4%.</t>
+          <t>EIMI.MI: scenario base Buy Watchlist, score 79.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 5.2%.</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -832,50 +832,50 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>47.345</v>
+        <v>47.26</v>
       </c>
       <c r="AA2" t="n">
         <v>69</v>
       </c>
       <c r="AB2" t="n">
-        <v>98.59999999999999</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="AC2" t="n">
         <v>65.5</v>
       </c>
       <c r="AD2" t="n">
-        <v>77.2</v>
+        <v>78</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.29</v>
+        <v>0.11</v>
       </c>
       <c r="AF2" t="n">
-        <v>25.07</v>
+        <v>24.84</v>
       </c>
       <c r="AG2" t="n">
-        <v>18.64</v>
+        <v>18.57</v>
       </c>
       <c r="AH2" t="n">
         <v>1.16</v>
       </c>
       <c r="AI2" t="n">
-        <v>44.9285</v>
+        <v>44.9268</v>
       </c>
       <c r="AJ2" t="n">
-        <v>40.3704</v>
+        <v>40.3699</v>
       </c>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="n">
         <v>85</v>
       </c>
       <c r="AM2" t="n">
-        <v>98.59999999999999</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="AN2" t="n">
         <v>65.5</v>
       </c>
       <c r="AO2" t="n">
-        <v>77.2</v>
+        <v>78</v>
       </c>
       <c r="AP2" t="n">
         <v>756</v>
@@ -893,10 +893,10 @@
         <v>49.485</v>
       </c>
       <c r="AU2" t="n">
-        <v>5.38</v>
+        <v>5.19</v>
       </c>
       <c r="AV2" t="n">
-        <v>17.28</v>
+        <v>17.07</v>
       </c>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
@@ -1176,10 +1176,10 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>10.51</v>
+        <v>10.45</v>
       </c>
       <c r="O4" t="n">
-        <v>24.27</v>
+        <v>24.21</v>
       </c>
       <c r="P4" t="n">
         <v>12.86</v>
@@ -1191,7 +1191,7 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 76.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.1%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 76.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.0%.</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1220,50 +1220,50 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>161.78</v>
+        <v>161.7</v>
       </c>
       <c r="AA4" t="n">
         <v>72.90000000000001</v>
       </c>
       <c r="AB4" t="n">
-        <v>78.09999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="AC4" t="n">
         <v>67.7</v>
       </c>
       <c r="AD4" t="n">
-        <v>82.40000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="AE4" t="n">
-        <v>1.99</v>
+        <v>1.94</v>
       </c>
       <c r="AF4" t="n">
-        <v>12.14</v>
+        <v>12.09</v>
       </c>
       <c r="AG4" t="n">
-        <v>17.23</v>
+        <v>17.21</v>
       </c>
       <c r="AH4" t="n">
         <v>1.34</v>
       </c>
       <c r="AI4" t="n">
-        <v>155.4288</v>
+        <v>155.4272</v>
       </c>
       <c r="AJ4" t="n">
-        <v>146.7651</v>
+        <v>146.7647</v>
       </c>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="n">
         <v>85</v>
       </c>
       <c r="AM4" t="n">
-        <v>78.09999999999999</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="AN4" t="n">
         <v>67.7</v>
       </c>
       <c r="AO4" t="n">
-        <v>82.40000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="AP4" t="n">
         <v>759</v>
@@ -1281,10 +1281,10 @@
         <v>164.88</v>
       </c>
       <c r="AU4" t="n">
-        <v>4.09</v>
+        <v>4.04</v>
       </c>
       <c r="AV4" t="n">
-        <v>10.23</v>
+        <v>10.18</v>
       </c>
       <c r="AW4" t="inlineStr"/>
       <c r="AX4" t="inlineStr"/>
@@ -1321,10 +1321,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>75.40000000000001</v>
+        <v>75.3</v>
       </c>
       <c r="G5" t="n">
-        <v>76</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1357,10 +1357,10 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>9.81</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="O5" t="n">
-        <v>22.25</v>
+        <v>22.22</v>
       </c>
       <c r="P5" t="n">
         <v>13.13</v>
@@ -1372,7 +1372,7 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 75.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 75.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>122.46</v>
+        <v>122.43</v>
       </c>
       <c r="AA5" t="n">
         <v>71.8</v>
       </c>
       <c r="AB5" t="n">
-        <v>75.5</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="AC5" t="n">
         <v>66.90000000000001</v>
@@ -1416,29 +1416,29 @@
         <v>82.8</v>
       </c>
       <c r="AE5" t="n">
-        <v>2.1</v>
+        <v>2.08</v>
       </c>
       <c r="AF5" t="n">
-        <v>10.28</v>
+        <v>10.26</v>
       </c>
       <c r="AG5" t="n">
-        <v>17.1</v>
+        <v>17.09</v>
       </c>
       <c r="AH5" t="n">
         <v>1.3</v>
       </c>
       <c r="AI5" t="n">
-        <v>117.9792</v>
+        <v>117.9786</v>
       </c>
       <c r="AJ5" t="n">
-        <v>112.2001</v>
+        <v>112.1999</v>
       </c>
       <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="n">
         <v>85</v>
       </c>
       <c r="AM5" t="n">
-        <v>75.5</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="AN5" t="n">
         <v>66.90000000000001</v>
@@ -1462,10 +1462,10 @@
         <v>124.27</v>
       </c>
       <c r="AU5" t="n">
-        <v>3.8</v>
+        <v>3.77</v>
       </c>
       <c r="AV5" t="n">
-        <v>9.140000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="AW5" t="inlineStr"/>
       <c r="AX5" t="inlineStr"/>
@@ -1502,7 +1502,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>74.5</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="G6" t="n">
         <v>75.40000000000001</v>
@@ -1538,10 +1538,10 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>6.87</v>
+        <v>6.78</v>
       </c>
       <c r="O6" t="n">
-        <v>15.88</v>
+        <v>15.79</v>
       </c>
       <c r="P6" t="n">
         <v>12.85</v>
@@ -1553,7 +1553,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.5%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.4%.</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1582,13 +1582,13 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>62.89</v>
+        <v>62.84</v>
       </c>
       <c r="AA6" t="n">
-        <v>70.3</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="AB6" t="n">
-        <v>69.90000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="AC6" t="n">
         <v>71.5</v>
@@ -1597,29 +1597,29 @@
         <v>82.8</v>
       </c>
       <c r="AE6" t="n">
-        <v>2.46</v>
+        <v>2.38</v>
       </c>
       <c r="AF6" t="n">
-        <v>10.57</v>
+        <v>10.48</v>
       </c>
       <c r="AG6" t="n">
-        <v>13.83</v>
+        <v>13.8</v>
       </c>
       <c r="AH6" t="n">
-        <v>1.08</v>
+        <v>1.07</v>
       </c>
       <c r="AI6" t="n">
-        <v>61.3456</v>
+        <v>61.3446</v>
       </c>
       <c r="AJ6" t="n">
-        <v>58.5817</v>
+        <v>58.5815</v>
       </c>
       <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="n">
         <v>85</v>
       </c>
       <c r="AM6" t="n">
-        <v>69.90000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="AN6" t="n">
         <v>71.5</v>
@@ -1643,10 +1643,10 @@
         <v>63.94</v>
       </c>
       <c r="AU6" t="n">
-        <v>2.52</v>
+        <v>2.44</v>
       </c>
       <c r="AV6" t="n">
-        <v>7.35</v>
+        <v>7.27</v>
       </c>
       <c r="AW6" t="inlineStr"/>
       <c r="AX6" t="inlineStr"/>
@@ -1719,10 +1719,10 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>11.07</v>
+        <v>11.06</v>
       </c>
       <c r="O7" t="n">
-        <v>23.42</v>
+        <v>23.41</v>
       </c>
       <c r="P7" t="n">
         <v>14.09</v>
@@ -1763,7 +1763,7 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>691.3200000000001</v>
+        <v>691.26</v>
       </c>
       <c r="AA7" t="n">
         <v>70.59999999999999</v>
@@ -1775,13 +1775,13 @@
         <v>64.40000000000001</v>
       </c>
       <c r="AD7" t="n">
-        <v>81.40000000000001</v>
+        <v>81.5</v>
       </c>
       <c r="AE7" t="n">
-        <v>2.11</v>
+        <v>2.1</v>
       </c>
       <c r="AF7" t="n">
-        <v>9.960000000000001</v>
+        <v>9.949999999999999</v>
       </c>
       <c r="AG7" t="n">
         <v>18.32</v>
@@ -1790,10 +1790,10 @@
         <v>1.3</v>
       </c>
       <c r="AI7" t="n">
-        <v>662.6455999999999</v>
+        <v>662.6444</v>
       </c>
       <c r="AJ7" t="n">
-        <v>629.989</v>
+        <v>629.9887</v>
       </c>
       <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="n">
@@ -1806,7 +1806,7 @@
         <v>64.40000000000001</v>
       </c>
       <c r="AO7" t="n">
-        <v>81.40000000000001</v>
+        <v>81.5</v>
       </c>
       <c r="AP7" t="n">
         <v>759</v>
@@ -1824,10 +1824,10 @@
         <v>703.9400000000001</v>
       </c>
       <c r="AU7" t="n">
-        <v>4.33</v>
+        <v>4.32</v>
       </c>
       <c r="AV7" t="n">
-        <v>9.74</v>
+        <v>9.73</v>
       </c>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
@@ -1900,10 +1900,10 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>7.42</v>
+        <v>7.39</v>
       </c>
       <c r="O8" t="n">
-        <v>18.04</v>
+        <v>18</v>
       </c>
       <c r="P8" t="n">
         <v>12.86</v>
@@ -1944,13 +1944,13 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>74.28</v>
+        <v>74.26000000000001</v>
       </c>
       <c r="AA8" t="n">
         <v>65</v>
       </c>
       <c r="AB8" t="n">
-        <v>70.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="AC8" t="n">
         <v>68.09999999999999</v>
@@ -1959,29 +1959,29 @@
         <v>82.8</v>
       </c>
       <c r="AE8" t="n">
-        <v>2.58</v>
+        <v>2.55</v>
       </c>
       <c r="AF8" t="n">
-        <v>9.69</v>
+        <v>9.66</v>
       </c>
       <c r="AG8" t="n">
-        <v>15.04</v>
+        <v>15.03</v>
       </c>
       <c r="AH8" t="n">
         <v>1.17</v>
       </c>
       <c r="AI8" t="n">
-        <v>71.908</v>
+        <v>71.9076</v>
       </c>
       <c r="AJ8" t="n">
-        <v>68.705</v>
+        <v>68.70489999999999</v>
       </c>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="n">
         <v>85</v>
       </c>
       <c r="AM8" t="n">
-        <v>70.7</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="AN8" t="n">
         <v>68.09999999999999</v>
@@ -2005,10 +2005,10 @@
         <v>74.95999999999999</v>
       </c>
       <c r="AU8" t="n">
-        <v>3.3</v>
+        <v>3.27</v>
       </c>
       <c r="AV8" t="n">
-        <v>8.109999999999999</v>
+        <v>8.09</v>
       </c>
       <c r="AW8" t="inlineStr"/>
       <c r="AX8" t="inlineStr"/>
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>79.2</v>
+        <v>79.3</v>
       </c>
       <c r="G12" t="n">
-        <v>65.59999999999999</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -2670,14 +2670,14 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>prezzo 11.7% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 11.5% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>28.04</v>
+        <v>27.84</v>
       </c>
       <c r="O12" t="n">
-        <v>61.97</v>
+        <v>61.72</v>
       </c>
       <c r="P12" t="n">
         <v>13.61</v>
@@ -2689,7 +2689,7 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Accumulate Carefully, score 79.2, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 11.7%.</t>
+          <t>XDEV.MI: scenario base Accumulate Carefully, score 79.3, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 11.5%.</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>70.91</v>
+        <v>70.8</v>
       </c>
       <c r="AA12" t="n">
         <v>79.09999999999999</v>
@@ -2730,25 +2730,25 @@
         <v>69.40000000000001</v>
       </c>
       <c r="AD12" t="n">
-        <v>51.9</v>
+        <v>52.6</v>
       </c>
       <c r="AE12" t="n">
-        <v>6.94</v>
+        <v>6.77</v>
       </c>
       <c r="AF12" t="n">
-        <v>38.39</v>
+        <v>38.17</v>
       </c>
       <c r="AG12" t="n">
-        <v>25.89</v>
+        <v>25.82</v>
       </c>
       <c r="AH12" t="n">
         <v>1.9</v>
       </c>
       <c r="AI12" t="n">
-        <v>63.4816</v>
+        <v>63.4794</v>
       </c>
       <c r="AJ12" t="n">
-        <v>54.8731</v>
+        <v>54.8726</v>
       </c>
       <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="n">
@@ -2761,7 +2761,7 @@
         <v>69.40000000000001</v>
       </c>
       <c r="AO12" t="n">
-        <v>51.9</v>
+        <v>52.6</v>
       </c>
       <c r="AP12" t="n">
         <v>756</v>
@@ -2779,10 +2779,10 @@
         <v>72.27</v>
       </c>
       <c r="AU12" t="n">
-        <v>11.7</v>
+        <v>11.53</v>
       </c>
       <c r="AV12" t="n">
-        <v>29.23</v>
+        <v>29.03</v>
       </c>
       <c r="AW12" t="inlineStr"/>
       <c r="AX12" t="inlineStr"/>
@@ -2819,10 +2819,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>68.90000000000001</v>
+        <v>69</v>
       </c>
       <c r="G13" t="n">
-        <v>64.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -2851,14 +2851,14 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>prezzo 9.4% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 9.3% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>28.95</v>
+        <v>28.86</v>
       </c>
       <c r="O13" t="n">
-        <v>40.03</v>
+        <v>39.94</v>
       </c>
       <c r="P13" t="n">
         <v>21.32</v>
@@ -2870,7 +2870,7 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Accumulate Carefully, score 68.9, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.4%.</t>
+          <t>RBOT.MI: scenario base Accumulate Carefully, score 69.0, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.3%.</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>17.692</v>
+        <v>17.68</v>
       </c>
       <c r="AA13" t="n">
         <v>51.3</v>
@@ -2911,22 +2911,22 @@
         <v>45.9</v>
       </c>
       <c r="AD13" t="n">
-        <v>61.1</v>
+        <v>61.4</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.95</v>
+        <v>0.88</v>
       </c>
       <c r="AF13" t="n">
-        <v>26.9</v>
+        <v>26.81</v>
       </c>
       <c r="AG13" t="n">
-        <v>17.88</v>
+        <v>17.86</v>
       </c>
       <c r="AH13" t="n">
         <v>0.84</v>
       </c>
       <c r="AI13" t="n">
-        <v>16.1688</v>
+        <v>16.1686</v>
       </c>
       <c r="AJ13" t="n">
         <v>14.4672</v>
@@ -2942,7 +2942,7 @@
         <v>50.9</v>
       </c>
       <c r="AO13" t="n">
-        <v>61.1</v>
+        <v>61.4</v>
       </c>
       <c r="AP13" t="n">
         <v>756</v>
@@ -2960,10 +2960,10 @@
         <v>18.17</v>
       </c>
       <c r="AU13" t="n">
-        <v>9.42</v>
+        <v>9.35</v>
       </c>
       <c r="AV13" t="n">
-        <v>22.29</v>
+        <v>22.21</v>
       </c>
       <c r="AW13" t="inlineStr"/>
       <c r="AX13" t="inlineStr"/>
@@ -3243,10 +3243,10 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>20.43</v>
+        <v>20.29</v>
       </c>
       <c r="O15" t="n">
-        <v>66.45999999999999</v>
+        <v>66.27</v>
       </c>
       <c r="P15" t="n">
         <v>23.17</v>
@@ -3258,7 +3258,7 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Hold / Monitor, score 64.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.9%.</t>
+          <t>INRG.MI: scenario base Hold / Monitor, score 64.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.7%.</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>10.574</v>
+        <v>10.562</v>
       </c>
       <c r="AA15" t="n">
         <v>31.2</v>
@@ -3302,19 +3302,19 @@
         <v>82.8</v>
       </c>
       <c r="AE15" t="n">
-        <v>-1.17</v>
+        <v>-1.28</v>
       </c>
       <c r="AF15" t="n">
-        <v>29.15</v>
+        <v>29.01</v>
       </c>
       <c r="AG15" t="n">
-        <v>3.26</v>
+        <v>3.22</v>
       </c>
       <c r="AH15" t="n">
         <v>0.14</v>
       </c>
       <c r="AI15" t="n">
-        <v>10.1818</v>
+        <v>10.1815</v>
       </c>
       <c r="AJ15" t="n">
         <v>8.756500000000001</v>
@@ -3348,10 +3348,10 @@
         <v>11.61</v>
       </c>
       <c r="AU15" t="n">
-        <v>3.85</v>
+        <v>3.74</v>
       </c>
       <c r="AV15" t="n">
-        <v>20.76</v>
+        <v>20.62</v>
       </c>
       <c r="AW15" t="inlineStr"/>
       <c r="AX15" t="inlineStr"/>
@@ -3631,16 +3631,16 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>-14.81</v>
+        <v>-14.77</v>
       </c>
       <c r="O17" t="n">
-        <v>27.66</v>
+        <v>27.72</v>
       </c>
       <c r="P17" t="n">
         <v>17.78</v>
       </c>
       <c r="Q17" t="n">
-        <v>-17.31</v>
+        <v>-17.28</v>
       </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 360.84 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 361.00 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -3675,13 +3675,13 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>360.84</v>
+        <v>361</v>
       </c>
       <c r="AA17" t="n">
         <v>70.59999999999999</v>
       </c>
       <c r="AB17" t="n">
-        <v>38.6</v>
+        <v>38.7</v>
       </c>
       <c r="AC17" t="n">
         <v>64.8</v>
@@ -3690,29 +3690,29 @@
         <v>67.40000000000001</v>
       </c>
       <c r="AE17" t="n">
-        <v>-6.65</v>
+        <v>-6.61</v>
       </c>
       <c r="AF17" t="n">
-        <v>4</v>
+        <v>4.05</v>
       </c>
       <c r="AG17" t="n">
-        <v>26.97</v>
+        <v>26.99</v>
       </c>
       <c r="AH17" t="n">
         <v>1.52</v>
       </c>
       <c r="AI17" t="n">
-        <v>380.8022</v>
+        <v>380.8054</v>
       </c>
       <c r="AJ17" t="n">
-        <v>362.1714</v>
+        <v>362.1722</v>
       </c>
       <c r="AK17" t="inlineStr"/>
       <c r="AL17" t="n">
         <v>35</v>
       </c>
       <c r="AM17" t="n">
-        <v>38.6</v>
+        <v>38.7</v>
       </c>
       <c r="AN17" t="n">
         <v>64.8</v>
@@ -3724,10 +3724,10 @@
         <v>756</v>
       </c>
       <c r="AQ17" t="n">
-        <v>360.84</v>
+        <v>361</v>
       </c>
       <c r="AR17" t="n">
-        <v>360.84</v>
+        <v>361</v>
       </c>
       <c r="AS17" t="n">
         <v>386.38</v>
@@ -3736,10 +3736,10 @@
         <v>424.57</v>
       </c>
       <c r="AU17" t="n">
-        <v>-5.24</v>
+        <v>-5.2</v>
       </c>
       <c r="AV17" t="n">
-        <v>-0.37</v>
+        <v>-0.32</v>
       </c>
       <c r="AW17" t="inlineStr"/>
       <c r="AX17" t="inlineStr"/>
@@ -4856,10 +4856,10 @@
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>61.9</v>
+        <v>62.1</v>
       </c>
       <c r="G24" t="n">
-        <v>18.9</v>
+        <v>20.2</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -4888,35 +4888,35 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>prezzo 18.6% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo 18.1% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="N24" t="n">
-        <v>33.76</v>
+        <v>33.27</v>
       </c>
       <c r="O24" t="n">
-        <v>128.18</v>
+        <v>127.34</v>
       </c>
       <c r="P24" t="n">
-        <v>38.11</v>
+        <v>38.1</v>
       </c>
       <c r="Q24" t="n">
         <v>-44.77</v>
       </c>
       <c r="R24" t="n">
-        <v>59.14</v>
+        <v>58.92</v>
       </c>
       <c r="S24" t="n">
-        <v>36.94</v>
+        <v>36.81</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 61.9, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.6%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 62.1, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.1%.</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 1531.60 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 1526.00 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -4936,29 +4936,29 @@
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="n">
-        <v>1531.6</v>
+        <v>1526</v>
       </c>
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
       <c r="AE24" t="n">
-        <v>17.31</v>
+        <v>16.88</v>
       </c>
       <c r="AF24" t="n">
-        <v>61.52</v>
+        <v>60.93</v>
       </c>
       <c r="AG24" t="n">
-        <v>32.66</v>
+        <v>32.5</v>
       </c>
       <c r="AH24" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="AI24" t="n">
-        <v>1291.7601</v>
+        <v>1291.6481</v>
       </c>
       <c r="AJ24" t="n">
-        <v>1052.333</v>
+        <v>1052.305</v>
       </c>
       <c r="AK24" t="inlineStr"/>
       <c r="AL24" t="n">
@@ -4971,7 +4971,7 @@
         <v>18.5</v>
       </c>
       <c r="AO24" t="n">
-        <v>24.5</v>
+        <v>26.2</v>
       </c>
       <c r="AP24" t="n">
         <v>765</v>
@@ -4983,16 +4983,16 @@
         <v>1109.5466</v>
       </c>
       <c r="AS24" t="n">
-        <v>1531.6</v>
+        <v>1526</v>
       </c>
       <c r="AT24" t="n">
-        <v>1531.6</v>
+        <v>1526</v>
       </c>
       <c r="AU24" t="n">
-        <v>18.57</v>
+        <v>18.14</v>
       </c>
       <c r="AV24" t="n">
-        <v>45.54</v>
+        <v>45.01</v>
       </c>
       <c r="AW24" t="inlineStr">
         <is>
@@ -5005,7 +5005,7 @@
         </is>
       </c>
       <c r="AY24" t="n">
-        <v>590305689600</v>
+        <v>588147326976</v>
       </c>
       <c r="AZ24" t="n">
         <v>29.71</v>
@@ -5029,13 +5029,13 @@
         <v>100</v>
       </c>
       <c r="BG24" t="n">
-        <v>11.5</v>
+        <v>11.7</v>
       </c>
       <c r="BH24" t="n">
         <v>18.5</v>
       </c>
       <c r="BI24" t="n">
-        <v>24.5</v>
+        <v>26.2</v>
       </c>
       <c r="BJ24" t="inlineStr"/>
       <c r="BK24" t="inlineStr">

</xml_diff>

<commit_message>
Apply AlphaForge patch: alpha_forge_v5_decision_portfolio_patch.zip
</commit_message>
<xml_diff>
--- a/AlphaForge_Insights.xlsx
+++ b/AlphaForge_Insights.xlsx
@@ -752,10 +752,10 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>79.3</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>79.8</v>
+        <v>79.7</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -788,13 +788,13 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>16.04</v>
+        <v>16.2</v>
       </c>
       <c r="O2" t="n">
-        <v>42.81</v>
+        <v>43</v>
       </c>
       <c r="P2" t="n">
-        <v>16</v>
+        <v>16.01</v>
       </c>
       <c r="Q2" t="n">
         <v>-19.17</v>
@@ -803,7 +803,7 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr">
         <is>
-          <t>EIMI.MI: scenario base Buy Watchlist, score 79.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 5.2%.</t>
+          <t>EIMI.MI: scenario base Buy Watchlist, score 79.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 5.3%.</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -832,50 +832,50 @@
         </is>
       </c>
       <c r="Z2" t="n">
-        <v>47.24</v>
+        <v>47.305</v>
       </c>
       <c r="AA2" t="n">
-        <v>69.09999999999999</v>
+        <v>69</v>
       </c>
       <c r="AB2" t="n">
-        <v>98</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="AC2" t="n">
         <v>65.5</v>
       </c>
       <c r="AD2" t="n">
-        <v>78.2</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.06</v>
+        <v>0.2</v>
       </c>
       <c r="AF2" t="n">
-        <v>24.79</v>
+        <v>24.96</v>
       </c>
       <c r="AG2" t="n">
-        <v>18.55</v>
+        <v>18.61</v>
       </c>
       <c r="AH2" t="n">
         <v>1.16</v>
       </c>
       <c r="AI2" t="n">
-        <v>44.9264</v>
+        <v>44.9277</v>
       </c>
       <c r="AJ2" t="n">
-        <v>40.3698</v>
+        <v>40.3702</v>
       </c>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="n">
         <v>85</v>
       </c>
       <c r="AM2" t="n">
-        <v>98</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="AN2" t="n">
         <v>65.5</v>
       </c>
       <c r="AO2" t="n">
-        <v>78.2</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AP2" t="n">
         <v>756</v>
@@ -893,10 +893,10 @@
         <v>49.485</v>
       </c>
       <c r="AU2" t="n">
-        <v>5.15</v>
+        <v>5.29</v>
       </c>
       <c r="AV2" t="n">
-        <v>17.02</v>
+        <v>17.18</v>
       </c>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
@@ -1143,7 +1143,7 @@
         <v>76.40000000000001</v>
       </c>
       <c r="G4" t="n">
-        <v>76.90000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1176,10 +1176,10 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>10.44</v>
+        <v>10.53</v>
       </c>
       <c r="O4" t="n">
-        <v>24.2</v>
+        <v>24.3</v>
       </c>
       <c r="P4" t="n">
         <v>12.86</v>
@@ -1191,7 +1191,7 @@
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr">
         <is>
-          <t>VWCE.DE: scenario base Accumulate Carefully, score 76.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.0%.</t>
+          <t>VWCE.DE: scenario base Accumulate Carefully, score 76.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.1%.</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1220,50 +1220,50 @@
         </is>
       </c>
       <c r="Z4" t="n">
-        <v>161.68</v>
+        <v>161.82</v>
       </c>
       <c r="AA4" t="n">
         <v>72.90000000000001</v>
       </c>
       <c r="AB4" t="n">
-        <v>77.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AC4" t="n">
         <v>67.7</v>
       </c>
       <c r="AD4" t="n">
-        <v>82.7</v>
+        <v>82.3</v>
       </c>
       <c r="AE4" t="n">
-        <v>1.93</v>
+        <v>2.02</v>
       </c>
       <c r="AF4" t="n">
-        <v>12.08</v>
+        <v>12.17</v>
       </c>
       <c r="AG4" t="n">
-        <v>17.2</v>
+        <v>17.23</v>
       </c>
       <c r="AH4" t="n">
         <v>1.34</v>
       </c>
       <c r="AI4" t="n">
-        <v>155.4268</v>
+        <v>155.4296</v>
       </c>
       <c r="AJ4" t="n">
-        <v>146.7646</v>
+        <v>146.7653</v>
       </c>
       <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="n">
         <v>85</v>
       </c>
       <c r="AM4" t="n">
-        <v>77.90000000000001</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="AN4" t="n">
         <v>67.7</v>
       </c>
       <c r="AO4" t="n">
-        <v>82.7</v>
+        <v>82.3</v>
       </c>
       <c r="AP4" t="n">
         <v>759</v>
@@ -1281,10 +1281,10 @@
         <v>164.88</v>
       </c>
       <c r="AU4" t="n">
-        <v>4.02</v>
+        <v>4.11</v>
       </c>
       <c r="AV4" t="n">
-        <v>10.16</v>
+        <v>10.26</v>
       </c>
       <c r="AW4" t="inlineStr"/>
       <c r="AX4" t="inlineStr"/>
@@ -1321,10 +1321,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>75.3</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="G5" t="n">
-        <v>75.90000000000001</v>
+        <v>76</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1357,10 +1357,10 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>9.77</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="O5" t="n">
-        <v>22.2</v>
+        <v>22.31</v>
       </c>
       <c r="P5" t="n">
         <v>13.13</v>
@@ -1372,7 +1372,7 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr">
         <is>
-          <t>SWDA.MI: scenario base Accumulate Carefully, score 75.3, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.8%.</t>
+          <t>SWDA.MI: scenario base Accumulate Carefully, score 75.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.9%.</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="Z5" t="n">
-        <v>122.41</v>
+        <v>122.52</v>
       </c>
       <c r="AA5" t="n">
         <v>71.8</v>
       </c>
       <c r="AB5" t="n">
-        <v>75.40000000000001</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="AC5" t="n">
         <v>66.90000000000001</v>
@@ -1416,29 +1416,29 @@
         <v>82.8</v>
       </c>
       <c r="AE5" t="n">
-        <v>2.06</v>
+        <v>2.15</v>
       </c>
       <c r="AF5" t="n">
-        <v>10.24</v>
+        <v>10.34</v>
       </c>
       <c r="AG5" t="n">
-        <v>17.09</v>
+        <v>17.12</v>
       </c>
       <c r="AH5" t="n">
         <v>1.3</v>
       </c>
       <c r="AI5" t="n">
-        <v>117.9782</v>
+        <v>117.9804</v>
       </c>
       <c r="AJ5" t="n">
-        <v>112.1999</v>
+        <v>112.2004</v>
       </c>
       <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="n">
         <v>85</v>
       </c>
       <c r="AM5" t="n">
-        <v>75.40000000000001</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="AN5" t="n">
         <v>66.90000000000001</v>
@@ -1462,10 +1462,10 @@
         <v>124.27</v>
       </c>
       <c r="AU5" t="n">
-        <v>3.76</v>
+        <v>3.85</v>
       </c>
       <c r="AV5" t="n">
-        <v>9.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AW5" t="inlineStr"/>
       <c r="AX5" t="inlineStr"/>
@@ -1502,7 +1502,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>74.40000000000001</v>
+        <v>74.5</v>
       </c>
       <c r="G6" t="n">
         <v>75.40000000000001</v>
@@ -1538,10 +1538,10 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>6.78</v>
+        <v>6.8</v>
       </c>
       <c r="O6" t="n">
-        <v>15.79</v>
+        <v>15.8</v>
       </c>
       <c r="P6" t="n">
         <v>12.85</v>
@@ -1553,7 +1553,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.4, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.4%.</t>
+          <t>EXSA.DE: scenario base Accumulate Carefully, score 74.5, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 2.5%.</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1582,13 +1582,13 @@
         </is>
       </c>
       <c r="Z6" t="n">
-        <v>62.84</v>
+        <v>62.85</v>
       </c>
       <c r="AA6" t="n">
         <v>70.09999999999999</v>
       </c>
       <c r="AB6" t="n">
-        <v>69.7</v>
+        <v>69.8</v>
       </c>
       <c r="AC6" t="n">
         <v>71.5</v>
@@ -1597,19 +1597,19 @@
         <v>82.8</v>
       </c>
       <c r="AE6" t="n">
-        <v>2.38</v>
+        <v>2.39</v>
       </c>
       <c r="AF6" t="n">
-        <v>10.48</v>
+        <v>10.5</v>
       </c>
       <c r="AG6" t="n">
-        <v>13.8</v>
+        <v>13.81</v>
       </c>
       <c r="AH6" t="n">
         <v>1.07</v>
       </c>
       <c r="AI6" t="n">
-        <v>61.3446</v>
+        <v>61.3448</v>
       </c>
       <c r="AJ6" t="n">
         <v>58.5815</v>
@@ -1619,7 +1619,7 @@
         <v>85</v>
       </c>
       <c r="AM6" t="n">
-        <v>69.7</v>
+        <v>69.8</v>
       </c>
       <c r="AN6" t="n">
         <v>71.5</v>
@@ -1643,10 +1643,10 @@
         <v>63.94</v>
       </c>
       <c r="AU6" t="n">
-        <v>2.44</v>
+        <v>2.45</v>
       </c>
       <c r="AV6" t="n">
-        <v>7.27</v>
+        <v>7.29</v>
       </c>
       <c r="AW6" t="inlineStr"/>
       <c r="AX6" t="inlineStr"/>
@@ -1686,7 +1686,7 @@
         <v>74.8</v>
       </c>
       <c r="G7" t="n">
-        <v>75.3</v>
+        <v>75.2</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1719,10 +1719,10 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>11.09</v>
+        <v>11.21</v>
       </c>
       <c r="O7" t="n">
-        <v>23.43</v>
+        <v>23.57</v>
       </c>
       <c r="P7" t="n">
         <v>14.09</v>
@@ -1734,7 +1734,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>SXR8.DE: scenario base Accumulate Carefully, score 74.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.3%.</t>
+          <t>SXR8.DE: scenario base Accumulate Carefully, score 74.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 4.5%.</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1763,50 +1763,50 @@
         </is>
       </c>
       <c r="Z7" t="n">
-        <v>691.4</v>
+        <v>692.16</v>
       </c>
       <c r="AA7" t="n">
         <v>70.59999999999999</v>
       </c>
       <c r="AB7" t="n">
-        <v>77.40000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AC7" t="n">
         <v>64.40000000000001</v>
       </c>
       <c r="AD7" t="n">
-        <v>81.40000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="AE7" t="n">
-        <v>2.12</v>
+        <v>2.23</v>
       </c>
       <c r="AF7" t="n">
-        <v>9.970000000000001</v>
+        <v>10.09</v>
       </c>
       <c r="AG7" t="n">
-        <v>18.33</v>
+        <v>18.37</v>
       </c>
       <c r="AH7" t="n">
         <v>1.3</v>
       </c>
       <c r="AI7" t="n">
-        <v>662.6472</v>
+        <v>662.6624</v>
       </c>
       <c r="AJ7" t="n">
-        <v>629.9894</v>
+        <v>629.9932</v>
       </c>
       <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="n">
         <v>85</v>
       </c>
       <c r="AM7" t="n">
-        <v>77.40000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AN7" t="n">
         <v>64.40000000000001</v>
       </c>
       <c r="AO7" t="n">
-        <v>81.40000000000001</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="AP7" t="n">
         <v>759</v>
@@ -1824,10 +1824,10 @@
         <v>703.9400000000001</v>
       </c>
       <c r="AU7" t="n">
-        <v>4.34</v>
+        <v>4.45</v>
       </c>
       <c r="AV7" t="n">
-        <v>9.75</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="AW7" t="inlineStr"/>
       <c r="AX7" t="inlineStr"/>
@@ -1864,10 +1864,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>72.7</v>
+        <v>72.8</v>
       </c>
       <c r="G8" t="n">
-        <v>74.2</v>
+        <v>74.3</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1900,10 +1900,10 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>7.39</v>
+        <v>7.49</v>
       </c>
       <c r="O8" t="n">
-        <v>18</v>
+        <v>18.12</v>
       </c>
       <c r="P8" t="n">
         <v>12.86</v>
@@ -1915,7 +1915,7 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>IWQU.MI: scenario base Accumulate Carefully, score 72.7, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.3%.</t>
+          <t>IWQU.MI: scenario base Accumulate Carefully, score 72.8, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 3.4%.</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1944,13 +1944,13 @@
         </is>
       </c>
       <c r="Z8" t="n">
-        <v>74.26000000000001</v>
+        <v>74.33</v>
       </c>
       <c r="AA8" t="n">
         <v>65</v>
       </c>
       <c r="AB8" t="n">
-        <v>70.59999999999999</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="AC8" t="n">
         <v>68.09999999999999</v>
@@ -1959,29 +1959,29 @@
         <v>82.8</v>
       </c>
       <c r="AE8" t="n">
-        <v>2.55</v>
+        <v>2.65</v>
       </c>
       <c r="AF8" t="n">
-        <v>9.66</v>
+        <v>9.76</v>
       </c>
       <c r="AG8" t="n">
-        <v>15.03</v>
+        <v>15.06</v>
       </c>
       <c r="AH8" t="n">
         <v>1.17</v>
       </c>
       <c r="AI8" t="n">
-        <v>71.9076</v>
+        <v>71.90900000000001</v>
       </c>
       <c r="AJ8" t="n">
-        <v>68.70489999999999</v>
+        <v>68.70529999999999</v>
       </c>
       <c r="AK8" t="inlineStr"/>
       <c r="AL8" t="n">
         <v>85</v>
       </c>
       <c r="AM8" t="n">
-        <v>70.59999999999999</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="AN8" t="n">
         <v>68.09999999999999</v>
@@ -2005,10 +2005,10 @@
         <v>74.95999999999999</v>
       </c>
       <c r="AU8" t="n">
-        <v>3.27</v>
+        <v>3.37</v>
       </c>
       <c r="AV8" t="n">
-        <v>8.09</v>
+        <v>8.19</v>
       </c>
       <c r="AW8" t="inlineStr"/>
       <c r="AX8" t="inlineStr"/>
@@ -2255,7 +2255,7 @@
         <v>68.2</v>
       </c>
       <c r="G10" t="n">
-        <v>70.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -2288,10 +2288,10 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>-2.02</v>
+        <v>-1.95</v>
       </c>
       <c r="O10" t="n">
-        <v>0.22</v>
+        <v>0.28</v>
       </c>
       <c r="P10" t="n">
         <v>9.56</v>
@@ -2303,7 +2303,7 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>MVOL.MI: scenario base Accumulate Carefully, score 68.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.6%.</t>
+          <t>MVOL.MI: scenario base Accumulate Carefully, score 68.2, trend Bullish. Entry zone: Constructive entry zone. Distanza da MA50: 0.7%.</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -2332,47 +2332,47 @@
         </is>
       </c>
       <c r="Z10" t="n">
-        <v>63.7</v>
+        <v>63.74</v>
       </c>
       <c r="AA10" t="n">
         <v>61.3</v>
       </c>
       <c r="AB10" t="n">
-        <v>48.1</v>
+        <v>48.2</v>
       </c>
       <c r="AC10" t="n">
-        <v>78.2</v>
+        <v>78.3</v>
       </c>
       <c r="AD10" t="n">
         <v>82.8</v>
       </c>
       <c r="AE10" t="n">
-        <v>2.64</v>
+        <v>2.71</v>
       </c>
       <c r="AF10" t="n">
-        <v>1.45</v>
+        <v>1.51</v>
       </c>
       <c r="AG10" t="n">
-        <v>6.55</v>
+        <v>6.57</v>
       </c>
       <c r="AH10" t="n">
         <v>0.6899999999999999</v>
       </c>
       <c r="AI10" t="n">
-        <v>63.3198</v>
+        <v>63.3206</v>
       </c>
       <c r="AJ10" t="n">
-        <v>63.1002</v>
+        <v>63.1004</v>
       </c>
       <c r="AK10" t="inlineStr"/>
       <c r="AL10" t="n">
         <v>85</v>
       </c>
       <c r="AM10" t="n">
-        <v>48.1</v>
+        <v>48.2</v>
       </c>
       <c r="AN10" t="n">
-        <v>78.2</v>
+        <v>78.3</v>
       </c>
       <c r="AO10" t="n">
         <v>82.8</v>
@@ -2393,10 +2393,10 @@
         <v>65.28</v>
       </c>
       <c r="AU10" t="n">
-        <v>0.6</v>
+        <v>0.66</v>
       </c>
       <c r="AV10" t="n">
-        <v>0.95</v>
+        <v>1.01</v>
       </c>
       <c r="AW10" t="inlineStr"/>
       <c r="AX10" t="inlineStr"/>
@@ -2638,10 +2638,10 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>79.3</v>
+        <v>79.2</v>
       </c>
       <c r="G12" t="n">
-        <v>66.09999999999999</v>
+        <v>65.5</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -2670,14 +2670,14 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>prezzo 11.5% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 11.7% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="N12" t="n">
-        <v>27.86</v>
+        <v>28.08</v>
       </c>
       <c r="O12" t="n">
-        <v>61.74</v>
+        <v>62.01</v>
       </c>
       <c r="P12" t="n">
         <v>13.61</v>
@@ -2689,7 +2689,7 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr">
         <is>
-          <t>XDEV.MI: scenario base Accumulate Carefully, score 79.3, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 11.6%.</t>
+          <t>XDEV.MI: scenario base Accumulate Carefully, score 79.2, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 11.7%.</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="Z12" t="n">
-        <v>70.81</v>
+        <v>70.93000000000001</v>
       </c>
       <c r="AA12" t="n">
         <v>79.09999999999999</v>
@@ -2730,25 +2730,25 @@
         <v>69.40000000000001</v>
       </c>
       <c r="AD12" t="n">
-        <v>52.6</v>
+        <v>51.8</v>
       </c>
       <c r="AE12" t="n">
-        <v>6.79</v>
+        <v>6.97</v>
       </c>
       <c r="AF12" t="n">
-        <v>38.19</v>
+        <v>38.43</v>
       </c>
       <c r="AG12" t="n">
-        <v>25.83</v>
+        <v>25.9</v>
       </c>
       <c r="AH12" t="n">
         <v>1.9</v>
       </c>
       <c r="AI12" t="n">
-        <v>63.4796</v>
+        <v>63.482</v>
       </c>
       <c r="AJ12" t="n">
-        <v>54.8726</v>
+        <v>54.8732</v>
       </c>
       <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="n">
@@ -2761,7 +2761,7 @@
         <v>69.40000000000001</v>
       </c>
       <c r="AO12" t="n">
-        <v>52.6</v>
+        <v>51.8</v>
       </c>
       <c r="AP12" t="n">
         <v>756</v>
@@ -2779,10 +2779,10 @@
         <v>72.27</v>
       </c>
       <c r="AU12" t="n">
-        <v>11.55</v>
+        <v>11.73</v>
       </c>
       <c r="AV12" t="n">
-        <v>29.04</v>
+        <v>29.26</v>
       </c>
       <c r="AW12" t="inlineStr"/>
       <c r="AX12" t="inlineStr"/>
@@ -2819,10 +2819,10 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>69</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="G13" t="n">
-        <v>65</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -2851,14 +2851,14 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>prezzo 9.3% sopra MA50: evitare inseguimento</t>
+          <t>prezzo 9.4% sopra MA50: evitare inseguimento</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>28.79</v>
+        <v>28.94</v>
       </c>
       <c r="O13" t="n">
-        <v>39.86</v>
+        <v>40.02</v>
       </c>
       <c r="P13" t="n">
         <v>21.32</v>
@@ -2870,7 +2870,7 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr">
         <is>
-          <t>RBOT.MI: scenario base Accumulate Carefully, score 69.0, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.3%.</t>
+          <t>RBOT.MI: scenario base Accumulate Carefully, score 68.9, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 9.4%.</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -2899,7 +2899,7 @@
         </is>
       </c>
       <c r="Z13" t="n">
-        <v>17.67</v>
+        <v>17.69</v>
       </c>
       <c r="AA13" t="n">
         <v>51.3</v>
@@ -2911,25 +2911,25 @@
         <v>45.9</v>
       </c>
       <c r="AD13" t="n">
-        <v>61.6</v>
+        <v>61.1</v>
       </c>
       <c r="AE13" t="n">
-        <v>0.82</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AF13" t="n">
-        <v>26.74</v>
+        <v>26.88</v>
       </c>
       <c r="AG13" t="n">
-        <v>17.83</v>
+        <v>17.88</v>
       </c>
       <c r="AH13" t="n">
         <v>0.84</v>
       </c>
       <c r="AI13" t="n">
-        <v>16.1684</v>
+        <v>16.1688</v>
       </c>
       <c r="AJ13" t="n">
-        <v>14.4671</v>
+        <v>14.4672</v>
       </c>
       <c r="AK13" t="inlineStr"/>
       <c r="AL13" t="n">
@@ -2942,7 +2942,7 @@
         <v>50.9</v>
       </c>
       <c r="AO13" t="n">
-        <v>61.6</v>
+        <v>61.1</v>
       </c>
       <c r="AP13" t="n">
         <v>756</v>
@@ -2960,10 +2960,10 @@
         <v>18.17</v>
       </c>
       <c r="AU13" t="n">
-        <v>9.289999999999999</v>
+        <v>9.41</v>
       </c>
       <c r="AV13" t="n">
-        <v>22.14</v>
+        <v>22.28</v>
       </c>
       <c r="AW13" t="inlineStr"/>
       <c r="AX13" t="inlineStr"/>
@@ -3243,10 +3243,10 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>20.29</v>
+        <v>20.41</v>
       </c>
       <c r="O15" t="n">
-        <v>66.27</v>
+        <v>66.43000000000001</v>
       </c>
       <c r="P15" t="n">
         <v>23.17</v>
@@ -3258,7 +3258,7 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr">
         <is>
-          <t>INRG.MI: scenario base Hold / Monitor, score 64.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.7%.</t>
+          <t>INRG.MI: scenario base Hold / Monitor, score 64.3, trend Bullish. Entry zone: Monitor / partial entry only. Distanza da MA50: 3.8%.</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="Z15" t="n">
-        <v>10.562</v>
+        <v>10.572</v>
       </c>
       <c r="AA15" t="n">
         <v>31.2</v>
@@ -3302,19 +3302,19 @@
         <v>82.8</v>
       </c>
       <c r="AE15" t="n">
-        <v>-1.28</v>
+        <v>-1.19</v>
       </c>
       <c r="AF15" t="n">
-        <v>29.01</v>
+        <v>29.13</v>
       </c>
       <c r="AG15" t="n">
-        <v>3.22</v>
+        <v>3.25</v>
       </c>
       <c r="AH15" t="n">
         <v>0.14</v>
       </c>
       <c r="AI15" t="n">
-        <v>10.1815</v>
+        <v>10.1817</v>
       </c>
       <c r="AJ15" t="n">
         <v>8.756500000000001</v>
@@ -3348,10 +3348,10 @@
         <v>11.61</v>
       </c>
       <c r="AU15" t="n">
-        <v>3.74</v>
+        <v>3.83</v>
       </c>
       <c r="AV15" t="n">
-        <v>20.62</v>
+        <v>20.73</v>
       </c>
       <c r="AW15" t="inlineStr"/>
       <c r="AX15" t="inlineStr"/>
@@ -3598,7 +3598,7 @@
         <v>55.6</v>
       </c>
       <c r="G17" t="n">
-        <v>57.3</v>
+        <v>57.4</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -3631,16 +3631,16 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>-14.85</v>
+        <v>-14.83</v>
       </c>
       <c r="O17" t="n">
-        <v>27.59</v>
+        <v>27.63</v>
       </c>
       <c r="P17" t="n">
         <v>17.78</v>
       </c>
       <c r="Q17" t="n">
-        <v>-17.36</v>
+        <v>-17.33</v>
       </c>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Scenario negativo: perdita area 360.64 o peggioramento trend; rischio attuale: Normal risk.</t>
+          <t>Scenario negativo: perdita area 360.75 o peggioramento trend; rischio attuale: Normal risk.</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -3675,10 +3675,10 @@
         </is>
       </c>
       <c r="Z17" t="n">
-        <v>360.64</v>
+        <v>360.75</v>
       </c>
       <c r="AA17" t="n">
-        <v>70.5</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="AB17" t="n">
         <v>38.5</v>
@@ -3687,25 +3687,25 @@
         <v>64.8</v>
       </c>
       <c r="AD17" t="n">
-        <v>67.3</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AE17" t="n">
-        <v>-6.7</v>
+        <v>-6.67</v>
       </c>
       <c r="AF17" t="n">
-        <v>3.95</v>
+        <v>3.98</v>
       </c>
       <c r="AG17" t="n">
-        <v>26.95</v>
+        <v>26.96</v>
       </c>
       <c r="AH17" t="n">
         <v>1.52</v>
       </c>
       <c r="AI17" t="n">
-        <v>380.7982</v>
+        <v>380.8004</v>
       </c>
       <c r="AJ17" t="n">
-        <v>362.1704</v>
+        <v>362.171</v>
       </c>
       <c r="AK17" t="inlineStr"/>
       <c r="AL17" t="n">
@@ -3718,16 +3718,16 @@
         <v>64.8</v>
       </c>
       <c r="AO17" t="n">
-        <v>67.3</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AP17" t="n">
         <v>756</v>
       </c>
       <c r="AQ17" t="n">
-        <v>360.64</v>
+        <v>360.75</v>
       </c>
       <c r="AR17" t="n">
-        <v>360.64</v>
+        <v>360.75</v>
       </c>
       <c r="AS17" t="n">
         <v>386.38</v>
@@ -3736,10 +3736,10 @@
         <v>424.57</v>
       </c>
       <c r="AU17" t="n">
-        <v>-5.29</v>
+        <v>-5.27</v>
       </c>
       <c r="AV17" t="n">
-        <v>-0.42</v>
+        <v>-0.39</v>
       </c>
       <c r="AW17" t="inlineStr"/>
       <c r="AX17" t="inlineStr"/>
@@ -4678,7 +4678,7 @@
         <v>37.7</v>
       </c>
       <c r="G23" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -4711,10 +4711,10 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>7.73</v>
+        <v>7.67</v>
       </c>
       <c r="O23" t="n">
-        <v>-15.21</v>
+        <v>-15.26</v>
       </c>
       <c r="P23" t="n">
         <v>33.93</v>
@@ -4755,34 +4755,34 @@
         </is>
       </c>
       <c r="Z23" t="n">
-        <v>26.89</v>
+        <v>26.875</v>
       </c>
       <c r="AA23" t="n">
         <v>22.4</v>
       </c>
       <c r="AB23" t="n">
-        <v>52.6</v>
+        <v>52.5</v>
       </c>
       <c r="AC23" t="n">
         <v>15.4</v>
       </c>
       <c r="AD23" t="n">
-        <v>51</v>
+        <v>51.2</v>
       </c>
       <c r="AE23" t="n">
-        <v>11.58</v>
+        <v>11.51</v>
       </c>
       <c r="AF23" t="n">
-        <v>-7.4</v>
+        <v>-7.46</v>
       </c>
       <c r="AG23" t="n">
-        <v>-1.96</v>
+        <v>-1.98</v>
       </c>
       <c r="AH23" t="n">
         <v>-0.06</v>
       </c>
       <c r="AI23" t="n">
-        <v>24.2648</v>
+        <v>24.2645</v>
       </c>
       <c r="AJ23" t="n">
         <v>26.9667</v>
@@ -4792,13 +4792,13 @@
         <v>55</v>
       </c>
       <c r="AM23" t="n">
-        <v>52.6</v>
+        <v>52.5</v>
       </c>
       <c r="AN23" t="n">
         <v>20.4</v>
       </c>
       <c r="AO23" t="n">
-        <v>51</v>
+        <v>51.2</v>
       </c>
       <c r="AP23" t="n">
         <v>757</v>
@@ -4816,10 +4816,10 @@
         <v>30.11</v>
       </c>
       <c r="AU23" t="n">
-        <v>10.82</v>
+        <v>10.76</v>
       </c>
       <c r="AV23" t="n">
-        <v>-0.28</v>
+        <v>-0.34</v>
       </c>
       <c r="AW23" t="inlineStr"/>
       <c r="AX23" t="inlineStr"/>
@@ -4856,10 +4856,10 @@
       </c>
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="n">
-        <v>62.2</v>
+        <v>62</v>
       </c>
       <c r="G24" t="n">
-        <v>20.7</v>
+        <v>19.8</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -4888,14 +4888,14 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>prezzo 18.0% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
+          <t>prezzo 18.3% sopra MA50: evitare inseguimento; vicino a resistenza 20D: attenzione a falso breakout</t>
         </is>
       </c>
       <c r="N24" t="n">
-        <v>33.09</v>
+        <v>33.42</v>
       </c>
       <c r="O24" t="n">
-        <v>127.04</v>
+        <v>127.61</v>
       </c>
       <c r="P24" t="n">
         <v>38.1</v>
@@ -4904,19 +4904,19 @@
         <v>-44.77</v>
       </c>
       <c r="R24" t="n">
-        <v>58.84</v>
+        <v>58.99</v>
       </c>
       <c r="S24" t="n">
-        <v>36.76</v>
+        <v>36.85</v>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>ASML.AS: scenario base Hold / Monitor, score 62.2, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.0%.</t>
+          <t>ASML.AS: scenario base Hold / Monitor, score 62.0, trend Bullish. Entry zone: Extended - wait pullback. Distanza da MA50: 18.3%.</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>Scenario positivo: conferma sopra area 1524.00 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
+          <t>Scenario positivo: conferma sopra area 1527.80 con momentum stabile; valutare solo se rischio e size restano coerenti.</t>
         </is>
       </c>
       <c r="V24" t="inlineStr">
@@ -4936,29 +4936,29 @@
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="n">
-        <v>1524</v>
+        <v>1527.8</v>
       </c>
       <c r="AA24" t="inlineStr"/>
       <c r="AB24" t="inlineStr"/>
       <c r="AC24" t="inlineStr"/>
       <c r="AD24" t="inlineStr"/>
       <c r="AE24" t="n">
-        <v>16.73</v>
+        <v>17.02</v>
       </c>
       <c r="AF24" t="n">
-        <v>60.72</v>
+        <v>61.12</v>
       </c>
       <c r="AG24" t="n">
-        <v>32.44</v>
+        <v>32.55</v>
       </c>
       <c r="AH24" t="n">
         <v>0.85</v>
       </c>
       <c r="AI24" t="n">
-        <v>1291.6081</v>
+        <v>1291.6841</v>
       </c>
       <c r="AJ24" t="n">
-        <v>1052.295</v>
+        <v>1052.314</v>
       </c>
       <c r="AK24" t="inlineStr"/>
       <c r="AL24" t="n">
@@ -4971,7 +4971,7 @@
         <v>18.5</v>
       </c>
       <c r="AO24" t="n">
-        <v>26.8</v>
+        <v>25.6</v>
       </c>
       <c r="AP24" t="n">
         <v>765</v>
@@ -4983,16 +4983,16 @@
         <v>1109.5466</v>
       </c>
       <c r="AS24" t="n">
-        <v>1524</v>
+        <v>1527.8</v>
       </c>
       <c r="AT24" t="n">
-        <v>1524</v>
+        <v>1527.8</v>
       </c>
       <c r="AU24" t="n">
-        <v>17.99</v>
+        <v>18.28</v>
       </c>
       <c r="AV24" t="n">
-        <v>44.83</v>
+        <v>45.18</v>
       </c>
       <c r="AW24" t="inlineStr">
         <is>
@@ -5005,7 +5005,7 @@
         </is>
       </c>
       <c r="AY24" t="n">
-        <v>587376492544</v>
+        <v>588841156608</v>
       </c>
       <c r="AZ24" t="n">
         <v>29.71</v>
@@ -5029,13 +5029,13 @@
         <v>100</v>
       </c>
       <c r="BG24" t="n">
-        <v>11.8</v>
+        <v>11.6</v>
       </c>
       <c r="BH24" t="n">
         <v>18.5</v>
       </c>
       <c r="BI24" t="n">
-        <v>26.8</v>
+        <v>25.6</v>
       </c>
       <c r="BJ24" t="inlineStr"/>
       <c r="BK24" t="inlineStr">

</xml_diff>